<commit_message>
feat(F-NAR-019): polish TREE-COL-011 xlsx
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-011.xlsx
+++ b/stories/arbres/TREE-COL-011.xlsx
@@ -2358,17 +2358,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Victorino sort les cubes, près du bac. Nina veut un mur, pour le tunnel. Le mur, d'abord ! Une table, pour le thermos ! Il empile trop vite. La pile penche. Un cube frappe le couvercle. Le pas se bloque. Victorino veut forcer. Il s'arrête. L'éclat de thermos est du mauvais côté. Je ne force pas. Tu regardes le couvercle ? L'éclat, oui. Nina pose son mur, cube après cube. Il attend, les cubes contre son genou. Le thermos reste fermé, lourd, tiède.</t>
+          <t>Victorino sort les cubes, près du bac. Nina veut un mur, pour le tunnel. Le mur, d'abord ! Une table, pour le thermos ! Il empile trop vite. La pile penche. Un cube frappe le couvercle. Le couvercle se bloque. Victorino veut forcer. Il s'arrête. L'éclat de thermos est du mauvais côté. Je ne force pas. Tu regardes le couvercle ? L'éclat, oui. Nina pose son mur, cube après cube. Il attend, les cubes contre son genou. Le thermos reste fermé, lourd, tiède.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino sort les cubes, près du bac. Nina veut un mur, pour le tunnel. Le mur, d'abord ! Une table, pour le thermos ! Il empile trop vite. La pile penche. Un cube frappe le couvercle. Le pas se bloque. Victorino veut forcer. Il s'arrête. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; est du mauvais côté. Je ne force pas. Tu regardes le couvercle ? L'éclat, oui. Nina pose son mur, cube après cube. Il attend, les cubes contre son genou. Le thermos reste fermé, lourd, tiède.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino sort les cubes, près du bac. Nina veut un mur, pour le tunnel. Le mur, d'abord ! Une table, pour le thermos ! Il empile trop vite. La pile penche. Un cube frappe le couvercle. Le couvercle se bloque. Victorino veut forcer. Il s'arrête. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; est du mauvais côté. Je ne force pas. Tu regardes le couvercle ? L'éclat, oui. Nina pose son mur, cube après cube. Il attend, les cubes contre son genou. Le thermos reste fermé, lourd, tiède.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Victorino sort les cubes, près du bac. Nina veut un mur, pour le tunnel. Le mur, d'abord ! Une table, pour le thermos ! Il empile trop vite. La pile penche. Un cube frappe le couvercle. Le pas se bloque. Victorino veut forcer. Il s'arrête. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; est du mauvais côté. Je ne force pas. Tu regardes le couvercle ? L'éclat, oui. Nina pose son mur, cube après cube. Il attend, les cubes contre son genou. Le thermos reste fermé, lourd, tiède.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino sort les cubes, près du bac. Nina veut un mur, pour le tunnel. Le mur, d'abord ! Une table, pour le thermos ! Il empile trop vite. La pile penche. Un cube frappe le couvercle. Le couvercle se bloque. Victorino veut forcer. Il s'arrête. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; est du mauvais côté. Je ne force pas. Tu regardes le couvercle ? L'éclat, oui. Nina pose son mur, cube après cube. Il attend, les cubes contre son genou. Le thermos reste fermé, lourd, tiède.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2513,7 +2513,7 @@
 narrateur|Il empile trop vite.
 narrateur|La pile penche.
 narrateur|Un cube frappe le couvercle.
-narrateur|Le pas se bloque.
+narrateur|Le couvercle se bloque.
 narrateur|Victorino veut forcer.
 narrateur|Il s'arrête.
 narrateur|L'éclat de thermos est du mauvais côté.
@@ -2750,17 +2750,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Nina pose le dernier cube du mur. Victorino tient l'ours contre le thermos. Lui, il goûte en premier ! L'ours garde mon tunnel ! Deux phrases, un seul ours. Il avance l'ours. Le mur tremble. Un cube tombe. Le thermos penche. Victorino s'arrête. Il refuse de foncer. Il tourne le couvercle vers l'éclat de thermos. Le pas cède, sans forcer. S'il te plaît, un coin, pour la soupe. Le coin près du bois, pas le tunnel. Il pose le thermos. L'éclat reste visible. Une seconde plus tard, le cube recouvrait tout.</t>
+          <t>Nina pose le dernier cube du mur. Victorino tient l'ours contre le thermos. Lui, il goûte en premier ! L'ours garde mon tunnel ! Deux phrases, un seul ours. Il avance l'ours. Le mur tremble. Un cube tombe. Le thermos penche. Victorino s'arrête. Il refuse de foncer. Il tourne le couvercle vers l'éclat de thermos. Le couvercle cède, sans forcer. S'il te plaît, un coin, pour la soupe. Le coin près du bois, pas le tunnel. Il pose le thermos. L'éclat reste visible. Une seconde plus tard, le cube recouvrait tout.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina pose le dernier cube du mur. Victorino tient l'ours contre le thermos. Lui, il goûte en premier ! L'ours garde mon tunnel ! Deux phrases, un seul ours. Il avance l'ours. Le mur tremble. Un cube tombe. Le thermos penche. Victorino s'arrête. Il refuse de foncer. Il tourne le couvercle vers l'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt;. Le pas cède, sans forcer. S'il te plaît, un coin, pour la soupe. Le coin près du bois, pas le tunnel. Il pose le thermos. L'éclat reste visible. Une seconde plus tard, le cube recouvrait tout.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina pose le dernier cube du mur. Victorino tient l'ours contre le thermos. Lui, il goûte en premier ! L'ours garde mon tunnel ! Deux phrases, un seul ours. Il avance l'ours. Le mur tremble. Un cube tombe. Le thermos penche. Victorino s'arrête. Il refuse de foncer. Il tourne le couvercle vers l'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt;. Le couvercle cède, sans forcer. S'il te plaît, un coin, pour la soupe. Le coin près du bois, pas le tunnel. Il pose le thermos. L'éclat reste visible. Une seconde plus tard, le cube recouvrait tout.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Nina pose le dernier cube du mur. Victorino tient l'ours contre le thermos. Lui, il goûte en premier ! L'ours garde mon tunnel ! Deux phrases, un seul ours. Il avance l'ours. Le mur tremble. Un cube tombe. Le thermos penche. Victorino s'arrête. Il refuse de foncer. Il tourne le couvercle vers l'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt;. Le pas cède, sans forcer. S'il te plaît, un coin, pour la soupe. Le coin près du bois, pas le tunnel. Il pose le thermos. L'éclat reste visible. Une seconde plus tard, le cube recouvrait tout. [pause]</t>
+          <t>Nina pose le dernier cube du mur. Victorino tient l'ours contre le thermos. Lui, il goûte en premier ! L'ours garde mon tunnel ! Deux phrases, un seul ours. Il avance l'ours. Le mur tremble. Un cube tombe. Le thermos penche. Victorino s'arrête. Il refuse de foncer. Il tourne le couvercle vers l'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt;. Le couvercle cède, sans forcer. S'il te plaît, un coin, pour la soupe. Le coin près du bois, pas le tunnel. Il pose le thermos. L'éclat reste visible. Une seconde plus tard, le cube recouvrait tout. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
 narrateur|Victorino s'arrête.
 narrateur|Il refuse de foncer.
 narrateur|Il tourne le couvercle vers l'éclat de thermos.
-narrateur|Le pas cède, sans forcer.
+narrateur|Le couvercle cède, sans forcer.
 enfant-m|S'il te plaît, un coin, pour la soupe.
 copine|Le coin près du bois, pas le tunnel.
 narrateur|Il pose le thermos.
@@ -5816,17 +5816,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Nina a sa tasse de sable, pleine. Victorino assied l'ours devant la dînette propre. Lui, il a la vraie ! La mienne, c'est la mer ! Il penche le thermos vers l'ours. Une goutte menace la tasse de sable. Il redresse. Il refuse de mélanger. L'éclat de thermos montre le bon sens. Il tourne. Le pas s'ouvre, net. S'il te plaît, une tasse vide. Celle-là, près de l'ours. Deux tasses, deux goûters. La soupe tombe dans le propre, pas dans le sable. L'ours a une goutte sur l'oreille, minuscule.</t>
+          <t>Nina a sa tasse de sable, pleine. Victorino assied l'ours devant la dînette propre. Lui, il a la vraie ! La mienne, c'est la mer ! Il penche le thermos vers l'ours. Une goutte menace la tasse de sable. Il redresse. Il refuse de mélanger. L'éclat de thermos montre le bon sens. Il tourne. Le couvercle s'ouvre, net. S'il te plaît, une tasse vide. Celle-là, près de l'ours. Deux tasses, deux goûters. La soupe tombe dans le propre, pas dans le sable. L'ours a une goutte sur l'oreille, minuscule.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina a sa tasse de sable, pleine. Victorino assied l'ours devant la dînette propre. Lui, il a la vraie ! La mienne, c'est la mer ! Il penche le thermos vers l'ours. Une goutte menace la tasse de sable. Il redresse. Il refuse de mélanger. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; montre le bon sens. Il tourne. Le pas s'ouvre, net. S'il te plaît, une tasse vide. Celle-là, près de l'ours. Deux tasses, deux goûters. La soupe tombe dans le propre, pas dans le sable. L'ours a une goutte sur l'oreille, minuscule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina a sa tasse de sable, pleine. Victorino assied l'ours devant la dînette propre. Lui, il a la vraie ! La mienne, c'est la mer ! Il penche le thermos vers l'ours. Une goutte menace la tasse de sable. Il redresse. Il refuse de mélanger. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; montre le bon sens. Il tourne. Le couvercle s'ouvre, net. S'il te plaît, une tasse vide. Celle-là, près de l'ours. Deux tasses, deux goûters. La soupe tombe dans le propre, pas dans le sable. L'ours a une goutte sur l'oreille, minuscule.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Nina a sa tasse de sable, pleine. Victorino assied l'ours devant la dînette propre. Lui, il a la vraie ! La mienne, c'est la mer ! Il penche le thermos vers l'ours. Une goutte menace la tasse de sable. Il redresse. Il refuse de mélanger. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; montre le bon sens. Il tourne. Le pas s'ouvre, net. S'il te plaît, une tasse vide. Celle-là, près de l'ours. Deux tasses, deux goûters. La soupe tombe dans le propre, pas dans le sable. L'ours a une goutte sur l'oreille, minuscule. [pause]</t>
+          <t>Nina a sa tasse de sable, pleine. Victorino assied l'ours devant la dînette propre. Lui, il a la vraie ! La mienne, c'est la mer ! Il penche le thermos vers l'ours. Une goutte menace la tasse de sable. Il redresse. Il refuse de mélanger. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; montre le bon sens. Il tourne. Le couvercle s'ouvre, net. S'il te plaît, une tasse vide. Celle-là, près de l'ours. Deux tasses, deux goûters. La soupe tombe dans le propre, pas dans le sable. L'ours a une goutte sur l'oreille, minuscule. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5970,7 +5970,7 @@
 narrateur|Il refuse de mélanger.
 narrateur|L'éclat de thermos montre le bon sens.
 narrateur|Il tourne.
-narrateur|Le pas s'ouvre, net.
+narrateur|Le couvercle s'ouvre, net.
 enfant-m|S'il te plaît, une tasse vide.
 copine|Celle-là, près de l'ours.
 papa|Deux tasses, deux goûters.
@@ -9057,17 +9057,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>La rampe est vide. La voix a changé de jeu. Deux cubes restent, comme des marches oubliées. L'éclat de thermos a pris la lumière du zinc, très loin. Tu n'as pas crié ? Non. J'ai glissé, sans bousculade. On reprend le quai, les mains libres ? Le thermos est moins lourd. Le toit de la gare cligne, au bout des rails. L'éclat cligne avec lui, plus près.</t>
+          <t>La rampe est vide. La voix a changé de jeu. Deux cubes restent, trop petits pour les pieds. L'éclat de thermos a pris la lumière du zinc, très loin. Tu n'as pas crié ? Non. J'ai glissé, sans bousculade. On reprend le quai, les mains libres ? Le thermos est moins lourd. Le toit de la gare cligne, au bout des rails. L'éclat cligne avec lui, plus près.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rampe est vide. La voix a changé de jeu. Deux cubes restent, comme des marches oubliées. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; a pris la lumière du zinc, très loin. Tu n'as pas crié ? Non. J'ai glissé, sans bousculade. On reprend le quai, les mains libres ? Le thermos est moins lourd. Le toit de la gare cligne, au bout des rails. L'éclat cligne avec lui, plus près.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rampe est vide. La voix a changé de jeu. Deux cubes restent, trop petits pour les pieds. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; a pris la lumière du zinc, très loin. Tu n'as pas crié ? Non. J'ai glissé, sans bousculade. On reprend le quai, les mains libres ? Le thermos est moins lourd. Le toit de la gare cligne, au bout des rails. L'éclat cligne avec lui, plus près.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rampe est vide. La voix a changé de jeu. Deux cubes restent, comme des marches oubliées. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; a pris la lumière du zinc, très loin. Tu n'as pas crié ? Non. J'ai glissé, sans bousculade. On reprend le quai, les mains libres ? Le thermos est moins lourd. Le toit de la gare cligne, au bout des rails. L'éclat cligne avec lui, plus près.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rampe est vide. La voix a changé de jeu. Deux cubes restent, trop petits pour les pieds. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; a pris la lumière du zinc, très loin. Tu n'as pas crié ? Non. J'ai glissé, sans bousculade. On reprend le quai, les mains libres ? Le thermos est moins lourd. Le toit de la gare cligne, au bout des rails. L'éclat cligne avec lui, plus près.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9207,7 +9207,7 @@
         <is>
           <t>narrateur|La rampe est vide.
 narrateur|La voix a changé de jeu.
-narrateur|Deux cubes restent, comme des marches oubliées.
+narrateur|Deux cubes restent, trop petits pour les pieds.
 narrateur|L'éclat de thermos a pris la lumière du zinc, très loin.
 papa|Tu n'as pas crié ?
 enfant-m|Non.
@@ -10211,17 +10211,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Nina referme le livre, à la fille qui glisse. Un coin de page est chaud, sous son pouce. L'éclat de thermos a un point de soupe, tout rond. Les deux tours sont passés ? Sa page, puis ma tasse. Puis le train. On file, le dessin au sec ? Oui. Le toit de la gare se penche dans la vitre du souvenir. L'éclat le recopie, cuivre sur métal.</t>
+          <t>Nina referme le livre, à la fille qui glisse. Un coin de page est chaud, sous son pouce. L'éclat de thermos a un point de soupe, tout rond. Les deux tours sont passés ? Sa page, puis ma tasse. Puis le train. On file, le dessin au sec ? Oui. Le toit de la gare se penche dans une flaque. L'éclat le recopie, cuivre sur métal.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina referme le livre, à la fille qui glisse. Un coin de page est chaud, sous son pouce. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; a un point de soupe, tout rond. Les deux tours sont passés ? Sa page, puis ma tasse. Puis le train. On file, le dessin au sec ? Oui. Le toit de la gare se penche dans la vitre du souvenir. L'éclat le recopie, cuivre sur métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina referme le livre, à la fille qui glisse. Un coin de page est chaud, sous son pouce. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; a un point de soupe, tout rond. Les deux tours sont passés ? Sa page, puis ma tasse. Puis le train. On file, le dessin au sec ? Oui. Le toit de la gare se penche dans une flaque. L'éclat le recopie, cuivre sur métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina referme le livre, à la fille qui glisse. Un coin de page est chaud, sous son pouce. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; a un point de soupe, tout rond. Les deux tours sont passés ? Sa page, puis ma tasse. Puis le train. On file, le dessin au sec ? Oui. Le toit de la gare se penche dans la vitre du souvenir. L'éclat le recopie, cuivre sur métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina referme le livre, à la fille qui glisse. Un coin de page est chaud, sous son pouce. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; a un point de soupe, tout rond. Les deux tours sont passés ? Sa page, puis ma tasse. Puis le train. On file, le dessin au sec ? Oui. Le toit de la gare se penche dans une flaque. L'éclat le recopie, cuivre sur métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10367,7 +10367,7 @@
 copine|Puis le train.
 maman|On file, le dessin au sec ?
 enfant-m|Oui.
-narrateur|Le toit de la gare se penche dans la vitre du souvenir.
+narrateur|Le toit de la gare se penche dans une flaque.
 narrateur|L'éclat le recopie, cuivre sur métal.</t>
         </is>
       </c>
@@ -11742,17 +11742,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le dessin de la tasse reste sec, sur l'herbe. La vraie tasse a un rond orange, au fond. L'éclat de thermos s'y mire, puis s'en va. Sa phrase était finie ? Oui. La ronde, comme la mienne. On file, avant que le métal refroidisse ? Il est tiède. Le zinc, au loin, n'a plus de goutte à offrir. L'éclat, lui, a servi.</t>
+          <t>Le dessin de la tasse reste sec, sur l'herbe. La vraie tasse a un rond orange, au fond. L'éclat de thermos s'y mire, puis s'en va. Sa phrase était finie ? Oui. La ronde, comme la mienne. On file, avant que le métal refroidisse ? Il est tiède. Le zinc, au loin, n'a plus de goutte à offrir. L'éclat reste, cuivre, sur le doigt.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le dessin de la tasse reste sec, sur l'herbe. La vraie tasse a un rond orange, au fond. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; s'y mire, puis s'en va. Sa phrase était finie ? Oui. La ronde, comme la mienne. On file, avant que le métal refroidisse ? Il est tiède. Le zinc, au loin, n'a plus de goutte à offrir. L'éclat, lui, a servi.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le dessin de la tasse reste sec, sur l'herbe. La vraie tasse a un rond orange, au fond. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; s'y mire, puis s'en va. Sa phrase était finie ? Oui. La ronde, comme la mienne. On file, avant que le métal refroidisse ? Il est tiède. Le zinc, au loin, n'a plus de goutte à offrir. L'éclat reste, cuivre, sur le doigt.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le dessin de la tasse reste sec, sur l'herbe. La vraie tasse a un rond orange, au fond. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; s'y mire, puis s'en va. Sa phrase était finie ? Oui. La ronde, comme la mienne. On file, avant que le métal refroidisse ? Il est tiède. Le zinc, au loin, n'a plus de goutte à offrir. L'éclat, lui, a servi.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le dessin de la tasse reste sec, sur l'herbe. La vraie tasse a un rond orange, au fond. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; s'y mire, puis s'en va. Sa phrase était finie ? Oui. La ronde, comme la mienne. On file, avant que le métal refroidisse ? Il est tiède. Le zinc, au loin, n'a plus de goutte à offrir. L'éclat reste, cuivre, sur le doigt.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11899,7 +11899,7 @@
 maman|On file, avant que le métal refroidisse ?
 enfant-m|Il est tiède.
 narrateur|Le zinc, au loin, n'a plus de goutte à offrir.
-narrateur|L'éclat, lui, a servi.</t>
+narrateur|L'éclat reste, cuivre, sur le doigt.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -12123,17 +12123,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>La tasse ne reprend pas la rampe. La voix cherche un caillou, plus loin. L'éclat de thermos a deux lueurs, ciel et zinc. Tu t'es figé, juste à temps ? Oui. La tasse est à nous. On reprend le quai ? Oui. Le toit de la gare rend la goutte du début. L'éclat la reconnaît, et se tait.</t>
+          <t>La tasse ne reprend pas la rampe. La voix cherche un caillou, plus loin. L'éclat de thermos a deux lueurs, ciel et zinc. Tu t'es figé, juste à temps ? Oui. La tasse est à nous. On reprend le quai ? Oui. Le toit de la gare rend la goutte du début. L'éclat la prend, tout petit, puis se tait.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tasse ne reprend pas la rampe. La voix cherche un caillou, plus loin. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; a deux lueurs, ciel et zinc. Tu t'es figé, juste à temps ? Oui. La tasse est à nous. On reprend le quai ? Oui. Le toit de la gare rend la goutte du début. L'éclat la reconnaît, et se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tasse ne reprend pas la rampe. La voix cherche un caillou, plus loin. L'&lt;emphasis level="moderate"&gt;éclat de thermos&lt;/emphasis&gt; a deux lueurs, ciel et zinc. Tu t'es figé, juste à temps ? Oui. La tasse est à nous. On reprend le quai ? Oui. Le toit de la gare rend la goutte du début. L'éclat la prend, tout petit, puis se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tasse ne reprend pas la rampe. La voix cherche un caillou, plus loin. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; a deux lueurs, ciel et zinc. Tu t'es figé, juste à temps ? Oui. La tasse est à nous. On reprend le quai ? Oui. Le toit de la gare rend la goutte du début. L'éclat la reconnaît, et se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tasse ne reprend pas la rampe. La voix cherche un caillou, plus loin. L'&lt;emphasis&gt;éclat de thermos&lt;/emphasis&gt; a deux lueurs, ciel et zinc. Tu t'es figé, juste à temps ? Oui. La tasse est à nous. On reprend le quai ? Oui. Le toit de la gare rend la goutte du début. L'éclat la prend, tout petit, puis se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12280,7 +12280,7 @@
 maman|On reprend le quai ?
 enfant-m|Oui.
 narrateur|Le toit de la gare rend la goutte du début.
-narrateur|L'éclat la reconnaît, et se tait.</t>
+narrateur|L'éclat la prend, tout petit, puis se tait.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
@@ -17663,7 +17663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17776,6 +17776,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>